<commit_message>
Membuat dashboard peta persebaran usaha dengan filter kecamatan, skala usaha, dan dan kategori lapangan usaha, serta pencarian usaha berdasarkan nama usaha
</commit_message>
<xml_diff>
--- a/FALSE_prelist_SE2026_ekraf.xlsx
+++ b/FALSE_prelist_SE2026_ekraf.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O49"/>
+  <dimension ref="A1:P50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -504,6 +504,11 @@
           <t>email</t>
         </is>
       </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>kdkec</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -557,6 +562,7 @@
         <v>6282368780119</v>
       </c>
       <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -598,6 +604,7 @@
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -641,6 +648,7 @@
         <v>82370171803</v>
       </c>
       <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -682,6 +690,7 @@
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -729,6 +738,7 @@
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -770,6 +780,7 @@
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -811,6 +822,7 @@
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -856,6 +868,7 @@
           <t>sarifmatua@gmail.com</t>
         </is>
       </c>
+      <c r="P9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -901,6 +914,7 @@
           <t>perdanadicka@gmail.com</t>
         </is>
       </c>
+      <c r="P10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -952,6 +966,7 @@
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -993,6 +1008,7 @@
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1036,6 +1052,7 @@
         <v>81383551221</v>
       </c>
       <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1077,6 +1094,7 @@
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1120,6 +1138,7 @@
         <v>81267681145</v>
       </c>
       <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1161,6 +1180,7 @@
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1204,6 +1224,7 @@
         <v>6281365555335</v>
       </c>
       <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1257,6 +1278,7 @@
         <v>6285271017113</v>
       </c>
       <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1312,6 +1334,7 @@
           <t>pasaman.network@gmail.com</t>
         </is>
       </c>
+      <c r="P19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1353,6 +1376,7 @@
       <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1408,6 +1432,7 @@
           <t>halalsertifikasi91@gmail.com</t>
         </is>
       </c>
+      <c r="P21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1459,6 +1484,7 @@
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1500,6 +1526,7 @@
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr"/>
       <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1541,6 +1568,7 @@
       <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr"/>
       <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1596,6 +1624,7 @@
           <t>megacentral89@gmail.com</t>
         </is>
       </c>
+      <c r="P25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1637,6 +1666,7 @@
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1680,6 +1710,7 @@
         <v>82278793698</v>
       </c>
       <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1725,6 +1756,7 @@
           <t>golegalitas4januari2024@gmail.com</t>
         </is>
       </c>
+      <c r="P28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1766,6 +1798,7 @@
       <c r="M29" t="inlineStr"/>
       <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1807,6 +1840,7 @@
       <c r="M30" t="inlineStr"/>
       <c r="N30" t="inlineStr"/>
       <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1856,6 +1890,7 @@
           <t>sarifmatua@gmail.com</t>
         </is>
       </c>
+      <c r="P31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1897,6 +1932,7 @@
       <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1952,6 +1988,7 @@
           <t>oss@pnm.co.id</t>
         </is>
       </c>
+      <c r="P33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1993,6 +2030,7 @@
       <c r="M34" t="inlineStr"/>
       <c r="N34" t="inlineStr"/>
       <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2034,6 +2072,7 @@
       <c r="M35" t="inlineStr"/>
       <c r="N35" t="inlineStr"/>
       <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2089,6 +2128,7 @@
           <t>oss@pnm.co.id</t>
         </is>
       </c>
+      <c r="P36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2130,6 +2170,7 @@
       <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr"/>
       <c r="O37" t="inlineStr"/>
+      <c r="P37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2171,6 +2212,7 @@
       <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr"/>
       <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -2214,6 +2256,7 @@
         <v>82391498869</v>
       </c>
       <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -2255,6 +2298,7 @@
       <c r="M40" t="inlineStr"/>
       <c r="N40" t="inlineStr"/>
       <c r="O40" t="inlineStr"/>
+      <c r="P40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -2306,6 +2350,7 @@
       <c r="M41" t="inlineStr"/>
       <c r="N41" t="inlineStr"/>
       <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -2347,6 +2392,7 @@
       <c r="M42" t="inlineStr"/>
       <c r="N42" t="inlineStr"/>
       <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2388,27 +2434,28 @@
       <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr"/>
       <c r="O43" t="inlineStr"/>
+      <c r="P43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>37094259</v>
+        <v>60127139</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>penjahit bordir novita &lt;Novita sari&gt;</t>
+          <t>YESI CELL</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>jl manunggal aia manggih, RT 0/RW 0, Kabupaten Pasaman</t>
+          <t>223H+7W8, MALAMPAH</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>1309080005</v>
+        <v>1309071003</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>eyJpdiI6Ik1wL3RDOWhpMXR1aktGbWw4bUxuQ0E9PSIsInZhbHVlIjoiV0NkaTN3SXExbDZrajhiOFRocWw4UT09IiwibWFjIjoiODhhZjkwODZhYWQ1NGE5MTI2Mzg1YjVhZjViZDUzZTgxMzBkNTU0NGMyMjkwZjI2NjViYmQxMWYwNjEyNDg0YSIsInRhZyI6IiJ9</t>
+          <t>eyJpdiI6IkRhR1RDZ1NIaFJUb0FwRDV5K1VwSFE9PSIsInZhbHVlIjoiWlhKRWhXYVNWWExtL3hLaHV3L1Jqdz09IiwibWFjIjoiOGNhOTgyMzEyYjhjN2Q4MTc4Zjg3Y2I0MmQzZmZiNjhhNjY0M2ZiYjRkZDQwZTdlZjg5Y2M4MTMyOGE3MDdjMyIsInRhZyI6IiJ9</t>
         </is>
       </c>
       <c r="F44" t="inlineStr"/>
@@ -2421,35 +2468,36 @@
       </c>
       <c r="J44" t="inlineStr"/>
       <c r="K44" t="n">
-        <v>-7.8651251</v>
+        <v>0.0025659</v>
       </c>
       <c r="L44" t="n">
-        <v>110.1563823</v>
+        <v>100.0299148</v>
       </c>
       <c r="M44" t="inlineStr"/>
       <c r="N44" t="inlineStr"/>
       <c r="O44" t="inlineStr"/>
+      <c r="P44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>42826888</v>
+        <v>37094259</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>BINTANG PERDANA NETWORK</t>
+          <t>penjahit bordir novita &lt;Novita sari&gt;</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Jalan Labuah Panjang, Kabupaten Pasaman</t>
+          <t>jl manunggal aia manggih, RT 0/RW 0, Kabupaten Pasaman</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>1309070003</v>
+        <v>1309080005</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>eyJpdiI6IlllOWdPVGtFS2I2dEwxMjBpKzl0MWc9PSIsInZhbHVlIjoiS3VGMVJTRytYbzNGa3gzQjlvbVBiQT09IiwibWFjIjoiYzM3MzU2Y2Y2YzhmOGU5MDQ0MzkwMmMxMjhjYmM5MTdiM2JmOGViZWZjMDNkMDNhZmZhYzIwMmJiZmM3MjM4YiIsInRhZyI6IiJ9</t>
+          <t>eyJpdiI6Ik1wL3RDOWhpMXR1aktGbWw4bUxuQ0E9PSIsInZhbHVlIjoiV0NkaTN3SXExbDZrajhiOFRocWw4UT09IiwibWFjIjoiODhhZjkwODZhYWQ1NGE5MTI2Mzg1YjVhZjViZDUzZTgxMzBkNTU0NGMyMjkwZjI2NjViYmQxMWYwNjEyNDg0YSIsInRhZyI6IiJ9</t>
         </is>
       </c>
       <c r="F45" t="inlineStr"/>
@@ -2460,105 +2508,103 @@
           <t>UMK</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>OSS - Badan Usaha</t>
-        </is>
-      </c>
+      <c r="J45" t="inlineStr"/>
       <c r="K45" t="n">
-        <v>-6.2855248</v>
+        <v>-7.8651251</v>
       </c>
       <c r="L45" t="n">
-        <v>106.8413317</v>
+        <v>110.1563823</v>
       </c>
       <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr"/>
-      <c r="O45" t="inlineStr">
-        <is>
-          <t>perdanadicka@gmail.com</t>
-        </is>
-      </c>
+      <c r="O45" t="inlineStr"/>
+      <c r="P45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>41527109</v>
+        <v>42826888</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>SURYANI RAHMI - rahmi bordir</t>
+          <t>BINTANG PERDANA NETWORK</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>KP balai Jr Sawah Laweh , Kabupaten Pasaman</t>
+          <t>Jalan Labuah Panjang, Kabupaten Pasaman</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>1309072002</v>
+        <v>1309070003</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>eyJpdiI6InZDZEJ5UG52SkNmUFlLelZRUGprcmc9PSIsInZhbHVlIjoiNDZyOXdIKzAxVFRCSHJIVmFRSmlxdz09IiwibWFjIjoiMGI5Mjg1NmU5MTlmNDY5YjM1NGI0ZGRiY2ZhOTI0ZGI2ZGRmMjgwOTk1N2NhNjc0NTAyMDljYzdhODg3ZGZkZSIsInRhZyI6IiJ9</t>
-        </is>
-      </c>
-      <c r="F46" t="n">
-        <v>10750</v>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>Industri Makanan dan Masakan Olahan</t>
-        </is>
-      </c>
+          <t>eyJpdiI6IlllOWdPVGtFS2I2dEwxMjBpKzl0MWc9PSIsInZhbHVlIjoiS3VGMVJTRytYbzNGa3gzQjlvbVBiQT09IiwibWFjIjoiYzM3MzU2Y2Y2YzhmOGU5MDQ0MzkwMmMxMjhjYmM5MTdiM2JmOGViZWZjMDNkMDNhZmZhYzIwMmJiZmM3MjM4YiIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr">
         <is>
           <t>UMK</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr"/>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>OSS - Badan Usaha</t>
+        </is>
+      </c>
       <c r="K46" t="n">
-        <v>-0.4687959</v>
+        <v>-6.2855248</v>
       </c>
       <c r="L46" t="n">
-        <v>100.3990746</v>
+        <v>106.8413317</v>
       </c>
       <c r="M46" t="inlineStr"/>
       <c r="N46" t="inlineStr"/>
       <c r="O46" t="inlineStr">
         <is>
-          <t>se.rti.fikathal.al8@gmail.com</t>
-        </is>
-      </c>
+          <t>perdanadicka@gmail.com</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>37317662</v>
+        <v>41527109</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>JUALAN ONLINE &lt;al ghaisan hafiz&gt;</t>
+          <t>SURYANI RAHMI - rahmi bordir</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Durian sikunik, Jr. Parik , koto kaciak, RT 0/RW 0, Kabupaten Pasaman</t>
+          <t>KP balai Jr Sawah Laweh , Kabupaten Pasaman</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>1309070001</v>
+        <v>1309072002</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>eyJpdiI6IlMzQmFRQzI2WmNCRjNodDhtei9samc9PSIsInZhbHVlIjoiNnoyc3owTE5rZUhISVdtUHpadU1ydz09IiwibWFjIjoiNzdlMjgwODQ3ZTFiZjY4OWViYjFjOTUwZWExYjQ3NDNlN2I3ZGNlOWNjNDQ4MWY2OGFkNzQyZWNkN2I4MjVjMyIsInRhZyI6IiJ9</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
+          <t>eyJpdiI6InZDZEJ5UG52SkNmUFlLelZRUGprcmc9PSIsInZhbHVlIjoiNDZyOXdIKzAxVFRCSHJIVmFRSmlxdz09IiwibWFjIjoiMGI5Mjg1NmU5MTlmNDY5YjM1NGI0ZGRiY2ZhOTI0ZGI2ZGRmMjgwOTk1N2NhNjc0NTAyMDljYzdhODg3ZGZkZSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>10750</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Industri Makanan dan Masakan Olahan</t>
+        </is>
+      </c>
       <c r="I47" t="inlineStr">
         <is>
           <t>UMK</t>
@@ -2566,52 +2612,45 @@
       </c>
       <c r="J47" t="inlineStr"/>
       <c r="K47" t="n">
-        <v>-7.7257966</v>
+        <v>-0.4687959</v>
       </c>
       <c r="L47" t="n">
-        <v>110.2640734</v>
+        <v>100.3990746</v>
       </c>
       <c r="M47" t="inlineStr"/>
-      <c r="N47" t="n">
-        <v>81263307179</v>
-      </c>
-      <c r="O47" t="inlineStr"/>
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>se.rti.fikathal.al8@gmail.com</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>41531760</v>
+        <v>37317662</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>PASAMAN KREATIF MEDIA - Pasaman Kreatif Media</t>
+          <t>JUALAN ONLINE &lt;al ghaisan hafiz&gt;</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Jalan Baru Terminal Benteng, Tanjuang Baringin, Kabupaten Pasaman</t>
+          <t>Durian sikunik, Jr. Parik , koto kaciak, RT 0/RW 0, Kabupaten Pasaman</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>1309080001</v>
+        <v>1309070001</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>eyJpdiI6Ilo4V3FiaVdoakF3M09xSEpPUCtoR2c9PSIsInZhbHVlIjoiaUFjTlFna3Zqa1pIWmVFbExEMUVxUT09IiwibWFjIjoiNWNjZGZmZjUzOWQ5MWEwZDJmMGYwNzc1ZmE0Y2VhNzY2NTJmOTcwNGFmNjAxOWEwY2ZiN2E0MjU1NDQwYzgwOCIsInRhZyI6IiJ9</t>
-        </is>
-      </c>
-      <c r="F48" t="n">
-        <v>73100</v>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>Periklanan</t>
-        </is>
-      </c>
+          <t>eyJpdiI6IlMzQmFRQzI2WmNCRjNodDhtei9samc9PSIsInZhbHVlIjoiNnoyc3owTE5rZUhISVdtUHpadU1ydz09IiwibWFjIjoiNzdlMjgwODQ3ZTFiZjY4OWViYjFjOTUwZWExYjQ3NDNlN2I3ZGNlOWNjNDQ4MWY2OGFkNzQyZWNkN2I4MjVjMyIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr">
         <is>
           <t>UMK</t>
@@ -2619,44 +2658,53 @@
       </c>
       <c r="J48" t="inlineStr"/>
       <c r="K48" t="n">
-        <v>0.1649365</v>
+        <v>-7.7257966</v>
       </c>
       <c r="L48" t="n">
-        <v>100.0543734</v>
+        <v>110.2640734</v>
       </c>
       <c r="M48" t="inlineStr"/>
-      <c r="N48" t="inlineStr"/>
-      <c r="O48" t="inlineStr">
-        <is>
-          <t>pasaman.network@gmail.com</t>
-        </is>
-      </c>
+      <c r="N48" t="n">
+        <v>81263307179</v>
+      </c>
+      <c r="O48" t="inlineStr"/>
+      <c r="P48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>37215941</v>
+        <v>41531760</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>KONTER HANAFI LUBIS &lt;HANAFI LUBIS&gt;</t>
+          <t>PASAMAN KREATIF MEDIA - Pasaman Kreatif Media</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>sontang, RT 0/RW 0</t>
+          <t>Jalan Baru Terminal Benteng, Tanjuang Baringin, Kabupaten Pasaman</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>1309111004</v>
+        <v>1309080001</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>eyJpdiI6ImVHenNNaEt4QzBMRlJzL2EzWW1CRWc9PSIsInZhbHVlIjoiWWJrUDVFdDRjdmprZ1owRTJ0Z2VBdz09IiwibWFjIjoiZmE4ZmU3MTUxNTI2Y2M5MzY4NmUzMTk4MDZhM2YxYTljMmRkYzAyNGE2MjlmZjNlN2EwM2Y0NzZmYWRhYmU1MCIsInRhZyI6IiJ9</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr"/>
-      <c r="H49" t="inlineStr"/>
+          <t>eyJpdiI6Ilo4V3FiaVdoakF3M09xSEpPUCtoR2c9PSIsInZhbHVlIjoiaUFjTlFna3Zqa1pIWmVFbExEMUVxUT09IiwibWFjIjoiNWNjZGZmZjUzOWQ5MWEwZDJmMGYwNzc1ZmE0Y2VhNzY2NTJmOTcwNGFmNjAxOWEwY2ZiN2E0MjU1NDQwYzgwOCIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>73100</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Periklanan</t>
+        </is>
+      </c>
       <c r="I49" t="inlineStr">
         <is>
           <t>UMK</t>
@@ -2664,16 +2712,63 @@
       </c>
       <c r="J49" t="inlineStr"/>
       <c r="K49" t="n">
+        <v>0.1649365</v>
+      </c>
+      <c r="L49" t="n">
+        <v>100.0543734</v>
+      </c>
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" t="inlineStr"/>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>pasaman.network@gmail.com</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>37215941</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>KONTER HANAFI LUBIS &lt;HANAFI LUBIS&gt;</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>sontang, RT 0/RW 0</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>1309111004</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>eyJpdiI6ImVHenNNaEt4QzBMRlJzL2EzWW1CRWc9PSIsInZhbHVlIjoiWWJrUDVFdDRjdmprZ1owRTJ0Z2VBdz09IiwibWFjIjoiZmE4ZmU3MTUxNTI2Y2M5MzY4NmUzMTk4MDZhM2YxYTljMmRkYzAyNGE2MjlmZjNlN2EwM2Y0NzZmYWRhYmU1MCIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>UMK</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="n">
         <v>5.5436714079664</v>
       </c>
-      <c r="L49" t="n">
+      <c r="L50" t="n">
         <v>95.30488003045301</v>
       </c>
-      <c r="M49" t="inlineStr"/>
-      <c r="N49" t="n">
+      <c r="M50" t="inlineStr"/>
+      <c r="N50" t="n">
         <v>82383446539</v>
       </c>
-      <c r="O49" t="inlineStr"/>
+      <c r="O50" t="inlineStr"/>
+      <c r="P50" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>